<commit_message>
Widen data columns to match reference, add brakerazh to breakfast
Columns without an explicit width (H onward for 22.08, I onward for 25.08)
now use the reference file's actual sheet-level default width (12.6328125)
instead of openpyxl's narrower fallback (~8.43), matching how the example
renders.

БРАКЕРАЖ (E) previously only appeared on обед/ужин main courses and was left
blank; it now also covers завтрак's three main dishes (каша/запеканка/омлет)
and E4 defaults to the order's stated brakerazh count as a starting estimate.
</commit_message>
<xml_diff>
--- a/output/Гонконг 22.08.2026 (обработка).xlsx
+++ b/output/Гонконг 22.08.2026 (обработка).xlsx
@@ -521,6 +521,21 @@
     <col width="15.88" customWidth="1" min="4" max="4"/>
     <col width="17.63" customWidth="1" min="5" max="5"/>
     <col width="14.63" customWidth="1" min="6" max="6"/>
+    <col width="14.63" customWidth="1" min="7" max="7"/>
+    <col width="12.6328125" customWidth="1" min="8" max="8"/>
+    <col width="12.6328125" customWidth="1" min="9" max="9"/>
+    <col width="12.6328125" customWidth="1" min="10" max="10"/>
+    <col width="12.6328125" customWidth="1" min="11" max="11"/>
+    <col width="12.6328125" customWidth="1" min="12" max="12"/>
+    <col width="12.6328125" customWidth="1" min="13" max="13"/>
+    <col width="12.6328125" customWidth="1" min="14" max="14"/>
+    <col width="12.6328125" customWidth="1" min="15" max="15"/>
+    <col width="12.6328125" customWidth="1" min="16" max="16"/>
+    <col width="12.6328125" customWidth="1" min="17" max="17"/>
+    <col width="12.6328125" customWidth="1" min="18" max="18"/>
+    <col width="12.6328125" customWidth="1" min="19" max="19"/>
+    <col width="12.6328125" customWidth="1" min="20" max="20"/>
+    <col width="12.6328125" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="32.25" customHeight="1">
@@ -828,7 +843,9 @@
       <c r="D4" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E4" s="9" t="n"/>
+      <c r="E4" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="F4" s="9" t="n">
         <v>1</v>
       </c>
@@ -989,7 +1006,10 @@
         <v/>
       </c>
       <c r="D6" s="15" t="n"/>
-      <c r="E6" s="15" t="n"/>
+      <c r="E6" s="15">
+        <f>E4</f>
+        <v/>
+      </c>
       <c r="F6" s="15" t="n"/>
       <c r="G6" s="15">
         <f>G4</f>
@@ -1094,7 +1114,10 @@
         <v/>
       </c>
       <c r="D8" s="15" t="n"/>
-      <c r="E8" s="15" t="n"/>
+      <c r="E8" s="15">
+        <f>E4</f>
+        <v/>
+      </c>
       <c r="F8" s="15" t="n"/>
       <c r="G8" s="15">
         <f>G4</f>
@@ -1190,7 +1213,10 @@
         <v/>
       </c>
       <c r="D10" s="15" t="n"/>
-      <c r="E10" s="15" t="n"/>
+      <c r="E10" s="15">
+        <f>E4</f>
+        <v/>
+      </c>
       <c r="F10" s="15" t="n"/>
       <c r="G10" s="15">
         <f>G4</f>

</xml_diff>